<commit_message>
return bacteria multifasta to original headers and remove from metadata
</commit_message>
<xml_diff>
--- a/assets/sample_metadata/Cdiphtheriae_test_1.xlsx
+++ b/assets/sample_metadata/Cdiphtheriae_test_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ick4\Downloads\kyle\updated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA441B6-1362-4084-A9C9-90293623D6A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1672C556-B784-4D71-A164-9E8DAC40727C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D029CB50-4CB9-4BD3-B61F-E5821D8D6205}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="79">
   <si>
     <t>Submission info</t>
   </si>
@@ -245,64 +245,34 @@
     <t>local</t>
   </si>
   <si>
-    <t>BX248355.1-segment2</t>
-  </si>
-  <si>
-    <t>BX248355.1-segment3</t>
-  </si>
-  <si>
-    <t>BX248355.1-segment4</t>
-  </si>
-  <si>
     <t>BBL-BIOINTEL</t>
   </si>
   <si>
-    <t>BX248355.1-segment2_Cd</t>
-  </si>
-  <si>
-    <t>BX248355.1-segment3_Cd</t>
-  </si>
-  <si>
-    <t>BX248355.1-segment4_Cd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BX248355.1-segment2 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BX248355.1-segment3 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BX248355.1-segment4 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">BX248355-1-segment4 </t>
-  </si>
-  <si>
     <t>fasta_path</t>
   </si>
   <si>
     <t>assets/sample_fastas/Cdiphtheriae/CP040557.fasta</t>
   </si>
   <si>
-    <t>assets/sample_fastas/Cdiphtheriae/BX248355.fasta</t>
-  </si>
-  <si>
     <t>assets/sample_fastqs/Cdiphtheriae/CP040557_R1.fastq.gz</t>
   </si>
   <si>
-    <t>assets/sample_fastqs/Cdiphtheriae/BX248355_R1.fastq.gz</t>
-  </si>
-  <si>
     <t>assets/sample_fastqs/Cdiphtheriae/CP040557_R2.fastq.gz</t>
   </si>
   <si>
-    <t>assets/sample_fastqs/Cdiphtheriae/BX248355_R2.fastq.gz</t>
-  </si>
-  <si>
-    <t>BX248355-1-segment3</t>
-  </si>
-  <si>
-    <t>BX248355-1-segment2</t>
+    <t>CP014051</t>
+  </si>
+  <si>
+    <t>assets/sample_fastas/Cdiphtheriae/CP014051.fasta</t>
+  </si>
+  <si>
+    <t>CP014051_Cd</t>
+  </si>
+  <si>
+    <t>assets/sample_fastqs/Cdiphtheriae/CP014051_R1.fastq.gz</t>
+  </si>
+  <si>
+    <t>assets/sample_fastqs/Cdiphtheriae/CP014051_R2.fastq.gz</t>
   </si>
 </sst>
 </file>
@@ -910,7 +880,7 @@
         <v>23</v>
       </c>
       <c r="AE2" s="5" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="AF2" s="6" t="s">
         <v>24</v>
@@ -982,7 +952,7 @@
         <v>62</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1" t="s">
@@ -1034,7 +1004,7 @@
       <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
       <c r="AE3" s="1" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="AF3" s="1" t="s">
         <v>67</v>
@@ -1049,10 +1019,10 @@
         <v>68</v>
       </c>
       <c r="AN3" s="1" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="AP3" s="1"/>
       <c r="AQ3" s="1"/>
@@ -1068,13 +1038,13 @@
     </row>
     <row r="4" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>88</v>
+        <v>74</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
@@ -1090,7 +1060,7 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>66</v>
@@ -1126,10 +1096,10 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
       <c r="AE4" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="AF4" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="AG4" s="1"/>
       <c r="AH4" s="1"/>
@@ -1141,10 +1111,10 @@
         <v>68</v>
       </c>
       <c r="AN4" s="1" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="1"/>
@@ -1159,56 +1129,28 @@
       <c r="AZ4" s="1"/>
     </row>
     <row r="5" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>72</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>65</v>
-      </c>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>66</v>
-      </c>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
-      <c r="O5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="R5" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
       <c r="S5" s="1"/>
-      <c r="T5" s="1" t="s">
-        <v>34</v>
-      </c>
+      <c r="T5" s="1"/>
       <c r="U5" s="1"/>
-      <c r="V5" s="1" t="s">
-        <v>34</v>
-      </c>
+      <c r="V5" s="1"/>
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
@@ -1217,27 +1159,17 @@
       <c r="AB5" s="1"/>
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
-      <c r="AE5" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="AF5" s="1" t="s">
-        <v>74</v>
-      </c>
+      <c r="AE5" s="1"/>
+      <c r="AF5" s="1"/>
       <c r="AG5" s="1"/>
       <c r="AH5" s="1"/>
       <c r="AI5" s="1"/>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="1"/>
       <c r="AL5" s="1"/>
-      <c r="AM5" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN5" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AO5" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="AM5" s="1"/>
+      <c r="AN5" s="1"/>
+      <c r="AO5" s="1"/>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="1"/>
       <c r="AR5" s="1"/>
@@ -1251,56 +1183,28 @@
       <c r="AZ5" s="1"/>
     </row>
     <row r="6" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>72</v>
-      </c>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
       <c r="D6" s="1"/>
-      <c r="E6" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>65</v>
-      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
-      <c r="K6" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>66</v>
-      </c>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
-      <c r="O6" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="R6" s="1" t="s">
-        <v>33</v>
-      </c>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
       <c r="S6" s="1"/>
-      <c r="T6" s="1" t="s">
-        <v>34</v>
-      </c>
+      <c r="T6" s="1"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="1" t="s">
-        <v>34</v>
-      </c>
+      <c r="V6" s="1"/>
       <c r="W6" s="1"/>
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
@@ -1309,27 +1213,17 @@
       <c r="AB6" s="1"/>
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
-      <c r="AE6" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="AF6" s="1" t="s">
-        <v>75</v>
-      </c>
+      <c r="AE6" s="1"/>
+      <c r="AF6" s="1"/>
       <c r="AG6" s="1"/>
       <c r="AH6" s="1"/>
       <c r="AI6" s="1"/>
       <c r="AJ6" s="1"/>
       <c r="AK6" s="1"/>
       <c r="AL6" s="1"/>
-      <c r="AM6" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN6" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="AO6" s="1" t="s">
-        <v>86</v>
-      </c>
+      <c r="AM6" s="1"/>
+      <c r="AN6" s="1"/>
+      <c r="AO6" s="1"/>
       <c r="AP6" s="1"/>
       <c r="AQ6" s="1"/>
       <c r="AR6" s="1"/>

</xml_diff>

<commit_message>
add required fields for OneHealth.1.0 BS package
</commit_message>
<xml_diff>
--- a/assets/sample_metadata/Cdiphtheriae_test_1.xlsx
+++ b/assets/sample_metadata/Cdiphtheriae_test_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ick4\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ick4\Downloads\sample_metadata2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E78F0DB9-D91D-4C1B-A1B8-ECFB378A45F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684298A4-AA03-479F-8DD9-E818F2D41274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5325" yWindow="2250" windowWidth="21600" windowHeight="11265" xr2:uid="{D029CB50-4CB9-4BD3-B61F-E5821D8D6205}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" xr2:uid="{D029CB50-4CB9-4BD3-B61F-E5821D8D6205}"/>
   </bookViews>
   <sheets>
     <sheet name="Diphtheria_Metadata" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="82">
   <si>
     <t>Submission info</t>
   </si>
@@ -273,13 +273,22 @@
   </si>
   <si>
     <t>BX248355</t>
+  </si>
+  <si>
+    <t>source_type</t>
+  </si>
+  <si>
+    <t>bs-package</t>
+  </si>
+  <si>
+    <t>strain</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -301,8 +310,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -313,6 +328,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF8FAADC"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF8FAADC"/>
       </patternFill>
     </fill>
   </fills>
@@ -381,7 +401,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -397,6 +417,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -714,13 +740,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43A21E4-DEDF-48C8-84DE-AC4607355643}">
-  <dimension ref="A1:AZ4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:BC4"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="47" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:55" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -788,7 +814,7 @@
       <c r="AY1" s="1"/>
       <c r="AZ1" s="1"/>
     </row>
-    <row r="2" spans="1:52" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:55" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -858,93 +884,102 @@
       <c r="W2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="X2" s="6" t="s">
+      <c r="X2" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="Y2" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="Z2" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="AB2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="AC2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="AA2" s="4" t="s">
+      <c r="AD2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="AB2" s="6" t="s">
+      <c r="AE2" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="AC2" s="4" t="s">
+      <c r="AF2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AD2" s="4" t="s">
+      <c r="AG2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="AE2" s="5" t="s">
+      <c r="AH2" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="AF2" s="6" t="s">
+      <c r="AI2" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AG2" s="6" t="s">
+      <c r="AJ2" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="AH2" s="4" t="s">
+      <c r="AK2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="AI2" s="4" t="s">
+      <c r="AL2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="AJ2" s="4" t="s">
+      <c r="AM2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="AK2" s="4" t="s">
+      <c r="AN2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="AL2" s="4" t="s">
+      <c r="AO2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="AM2" s="4" t="s">
+      <c r="AP2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="AN2" s="4" t="s">
+      <c r="AQ2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="AO2" s="4" t="s">
+      <c r="AR2" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="AP2" s="6" t="s">
+      <c r="AS2" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="AQ2" s="4" t="s">
+      <c r="AT2" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="AR2" s="4" t="s">
+      <c r="AU2" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AS2" s="4" t="s">
+      <c r="AV2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AT2" s="4" t="s">
+      <c r="AW2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="AU2" s="4" t="s">
+      <c r="AX2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="AV2" s="4" t="s">
+      <c r="AY2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="AW2" s="1"/>
-      <c r="AX2" s="4" t="s">
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="AY2" s="4" t="s">
+      <c r="BB2" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="AZ2" s="4" t="s">
+      <c r="BC2" s="4" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>62</v>
       </c>
@@ -1036,7 +1071,7 @@
       <c r="AY3" s="1"/>
       <c r="AZ3" s="1"/>
     </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>78</v>
       </c>

</xml_diff>